<commit_message>
Correct literature citations, regex gaps, remove GO:CC computation
- Remove incorrect citations: Robinson 2017 (not mTORC1/UPR),
  Schild 2015 (not ECM), Melov 2007 (not cytoskeletal reversal),
  MoTrPAC 2024 (not FCM). Themes now described as data-driven.
- Fix 3 regex false negatives: add coagulat (Theme 5), peroxide
  (Theme 7), actin (Theme 4). Themed proteins 756→775, Other 117→98.
- Remove GO:CC enrichment + rrvgo (computed then discarded).
- Fix stale "Top 3" comment in panel_C.R.
</commit_message>
<xml_diff>
--- a/04_Figures/F4/c_data/F4_supplementary.xlsx
+++ b/04_Figures/F4/c_data/F4_supplementary.xlsx
@@ -71881,7 +71881,7 @@
         <v>2279</v>
       </c>
       <c r="C4" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -71892,7 +71892,7 @@
         <v>2280</v>
       </c>
       <c r="C5" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -71977,10 +71977,10 @@
         <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>2279</v>
+        <v>2284</v>
       </c>
       <c r="C13" t="n">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14">
@@ -71988,10 +71988,10 @@
         <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>2284</v>
+        <v>2285</v>
       </c>
       <c r="C14" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15">
@@ -71999,10 +71999,10 @@
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>2285</v>
+        <v>2279</v>
       </c>
       <c r="C15" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
@@ -72010,9 +72010,20 @@
         <v>35</v>
       </c>
       <c r="B16" t="s">
+        <v>2283</v>
+      </c>
+      <c r="C16" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" t="s">
         <v>2278</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C17" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(F4): correct literature citations, regex gaps, remove GO:CC computation
- Remove incorrect citations: Robinson 2017 (not mTORC1/UPR),
  Schild 2015 (not ECM), Melov 2007 (not cytoskeletal reversal),
  MoTrPAC 2024 (not FCM). Themes now described as data-driven.
- Fix 3 regex false negatives: add coagulat (Theme 5), peroxide
  (Theme 7), actin (Theme 4). Themed proteins 756→775, Other 117→98.
- Remove GO:CC enrichment + rrvgo (computed then discarded).
- Fix stale "Top 3" comment in panel_C.R.
</commit_message>
<xml_diff>
--- a/04_Figures/F4/c_data/F4_supplementary.xlsx
+++ b/04_Figures/F4/c_data/F4_supplementary.xlsx
@@ -71881,7 +71881,7 @@
         <v>2279</v>
       </c>
       <c r="C4" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -71892,7 +71892,7 @@
         <v>2280</v>
       </c>
       <c r="C5" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -71977,10 +71977,10 @@
         <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>2279</v>
+        <v>2284</v>
       </c>
       <c r="C13" t="n">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14">
@@ -71988,10 +71988,10 @@
         <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>2284</v>
+        <v>2285</v>
       </c>
       <c r="C14" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15">
@@ -71999,10 +71999,10 @@
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>2285</v>
+        <v>2279</v>
       </c>
       <c r="C15" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
@@ -72010,9 +72010,20 @@
         <v>35</v>
       </c>
       <c r="B16" t="s">
+        <v>2283</v>
+      </c>
+      <c r="C16" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" t="s">
         <v>2278</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C17" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>